<commit_message>
Added the epics and user stories document and updated the functional requirements document
</commit_message>
<xml_diff>
--- a/Dokumentace/Funkcni_pozadavky_tankovani.xlsx
+++ b/Dokumentace/Funkcni_pozadavky_tankovani.xlsx
@@ -296,7 +296,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="52">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -377,6 +377,78 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -633,35 +705,41 @@
       <x:c r="C6" s="4"/>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
-      <x:c r="A7" s="7" t="str">
-        <x:v>FP-01</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="s">
+      <x:c r="A7" s="28" t="inlineStr">
+        <x:is>
+          <x:t>FP-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="29" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
+      <x:c r="C7" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
-      <x:c r="A8" s="10" t="str">
-        <x:v>FP-02</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="s">
+      <x:c r="A8" s="31" t="inlineStr">
+        <x:is>
+          <x:t>FP-02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="32" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="s">
+      <x:c r="C8" s="33" t="s">
         <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="59" customHeight="1">
-      <x:c r="A9" s="7" t="str">
-        <x:v>FP-03</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="s">
+      <x:c r="A9" s="28" t="inlineStr">
+        <x:is>
+          <x:t>FP-03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="29" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C9" s="6" t="s">
+      <x:c r="C9" s="30" t="s">
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -673,296 +751,388 @@
       <x:c r="C10" s="4"/>
     </x:row>
     <x:row r="11" ht="59" customHeight="1">
-      <x:c r="A11" s="10" t="str">
-        <x:v>FP-04</x:v>
-      </x:c>
-      <x:c r="B11" s="11" t="s">
+      <x:c r="A11" s="31" t="inlineStr">
+        <x:is>
+          <x:t>FP-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="32" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C11" s="9" t="s">
+      <x:c r="C11" s="33" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="46" customHeight="1">
-      <x:c r="A12" s="7" t="str">
-        <x:v>FP-05</x:v>
-      </x:c>
-      <x:c r="B12" s="8" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="str">
-        <x:v>U tankování musí být možné nepovinně zadat stav tachometru v kilometrech.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="46" customHeight="1">
-      <x:c r="A13" s="10" t="str">
-        <x:v>FP-06</x:v>
-      </x:c>
-      <x:c r="B13" s="11" t="s">
+    <x:row r="12" ht="59.0" customHeight="1">
+      <x:c r="A12" s="28" t="inlineStr">
+        <x:is>
+          <x:t>FP-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="29" t="inlineStr">
+        <x:is>
+          <x:t>Tachometr a tankování do plna</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Aplikace musí umožnit u tankování označit, zda bylo natankováno do plna. Stav tachometru v kilometrech musí být možné zadat nepovinně.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="59.0" customHeight="1">
+      <x:c r="A13" s="31" t="inlineStr">
+        <x:is>
+          <x:t>FP-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="32" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="s">
-        <x:v>17</x:v>
+      <x:c r="C13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Aplikace musí umožnit upravit údaje uloženého tankování, včetně změny označení tankování do plna a pozdějšího doplnění stavu tachometru a polohy.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
-      <x:c r="A14" s="7" t="str">
-        <x:v>FP-07</x:v>
-      </x:c>
-      <x:c r="B14" s="8" t="s">
+      <x:c r="A14" s="28" t="inlineStr">
+        <x:is>
+          <x:t>FP-07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="29" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="C14" s="6" t="s">
+      <x:c r="C14" s="30" t="s">
         <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
       <x:c r="A15" s="4"/>
-      <x:c r="B15" s="5" t="s">
-        <x:v>20</x:v>
+      <x:c r="B15" s="5" t="inlineStr">
+        <x:is>
+          <x:t>Fotografie a OCR</x:t>
+        </x:is>
       </x:c>
       <x:c r="C15" s="4"/>
     </x:row>
     <x:row r="16" ht="59" customHeight="1">
-      <x:c r="A16" s="10" t="str">
-        <x:v>FP-08</x:v>
-      </x:c>
-      <x:c r="B16" s="11" t="s">
+      <x:c r="A16" s="31" t="inlineStr">
+        <x:is>
+          <x:t>FP-08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="32" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C16" s="9" t="s">
+      <x:c r="C16" s="33" t="s">
         <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="59" customHeight="1">
-      <x:c r="A17" s="7" t="str">
-        <x:v>FP-09</x:v>
-      </x:c>
-      <x:c r="B17" s="8" t="s">
+      <x:c r="A17" s="28" t="inlineStr">
+        <x:is>
+          <x:t>FP-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="29" t="inlineStr">
+        <x:is>
+          <x:t>Načtení stavu tachometru z fotografie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Aplikace musí umožnit vyfotit stav celkového počtu ujetých kilometrů na displeji palubní desky a z fotografie předvyplnit stav tachometru v kilometrech do záznamu tankování.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="59" customHeight="1">
+      <x:c r="A18" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="35" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C17" s="6" t="s">
+      <x:c r="C18" s="36" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="59" customHeight="1">
-      <x:c r="A18" s="10" t="str">
-        <x:v>FP-10</x:v>
-      </x:c>
-      <x:c r="B18" s="11" t="s">
+    <x:row r="19" ht="59" customHeight="1">
+      <x:c r="A19" s="37" t="inlineStr">
+        <x:is>
+          <x:t>FP-11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="38" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C18" s="9" t="s">
+      <x:c r="C19" s="39" t="s">
         <x:v>26</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="59" customHeight="1">
-      <x:c r="A19" s="7" t="str">
-        <x:v>FP-11</x:v>
-      </x:c>
-      <x:c r="B19" s="8" t="s">
+    <x:row r="20" ht="59" customHeight="1">
+      <x:c r="A20" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="35" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="C19" s="6" t="s">
+      <x:c r="C20" s="36" t="s">
         <x:v>28</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="27" customHeight="1">
-      <x:c r="A20" s="4"/>
-      <x:c r="B20" s="5" t="s">
+    <x:row r="21" ht="27" customHeight="1">
+      <x:c r="A21" s="4"/>
+      <x:c r="B21" s="5" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="C20" s="4"/>
-    </x:row>
-    <x:row r="21" ht="59" customHeight="1">
-      <x:c r="A21" s="10" t="str">
-        <x:v>FP-12</x:v>
-      </x:c>
-      <x:c r="B21" s="11" t="s">
+      <x:c r="C21" s="4"/>
+    </x:row>
+    <x:row r="22" ht="59" customHeight="1">
+      <x:c r="A22" s="37" t="inlineStr">
+        <x:is>
+          <x:t>FP-13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="38" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C21" s="9" t="s">
+      <x:c r="C22" s="39" t="s">
         <x:v>31</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="46" customHeight="1">
-      <x:c r="A22" s="7" t="str">
-        <x:v>FP-13</x:v>
-      </x:c>
-      <x:c r="B22" s="8" t="s">
+    <x:row r="23" ht="46" customHeight="1">
+      <x:c r="A23" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="35" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C22" s="6" t="s">
+      <x:c r="C23" s="36" t="s">
         <x:v>33</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="59" customHeight="1">
-      <x:c r="A23" s="10" t="str">
-        <x:v>FP-14</x:v>
-      </x:c>
-      <x:c r="B23" s="11" t="s">
+    <x:row r="24" ht="59" customHeight="1">
+      <x:c r="A24" s="37" t="inlineStr">
+        <x:is>
+          <x:t>FP-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="38" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="C23" s="9" t="s">
+      <x:c r="C24" s="39" t="s">
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="27" customHeight="1">
-      <x:c r="A24" s="4"/>
-      <x:c r="B24" s="5" t="s">
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="A25" s="4"/>
+      <x:c r="B25" s="5" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="C24" s="4"/>
-    </x:row>
-    <x:row r="25" ht="59" customHeight="1">
-      <x:c r="A25" s="7" t="str">
-        <x:v>FP-15</x:v>
-      </x:c>
-      <x:c r="B25" s="8" t="s">
+      <x:c r="C25" s="4"/>
+    </x:row>
+    <x:row r="26" ht="59" customHeight="1">
+      <x:c r="A26" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="35" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C25" s="6" t="s">
+      <x:c r="C26" s="36" t="s">
         <x:v>38</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="59" customHeight="1">
-      <x:c r="A26" s="10" t="str">
-        <x:v>FP-16</x:v>
-      </x:c>
-      <x:c r="B26" s="11" t="s">
+    <x:row r="27" ht="59" customHeight="1">
+      <x:c r="A27" s="37" t="inlineStr">
+        <x:is>
+          <x:t>FP-17</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="38" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C26" s="9" t="s">
-        <x:v>40</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="27" customHeight="1">
-      <x:c r="A27" s="4"/>
-      <x:c r="B27" s="5" t="s">
+      <x:c r="C27" s="39" t="inlineStr">
+        <x:is>
+          <x:t>Aplikace musí umožnit otevřít záznam tankování a zobrazit všechny jeho uložené údaje včetně označení tankování do plna, polohy a stavu tachometru, pokud byly zadány.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="27" customHeight="1">
+      <x:c r="A28" s="4"/>
+      <x:c r="B28" s="5" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="C27" s="4"/>
-    </x:row>
-    <x:row r="28" ht="73" customHeight="1">
-      <x:c r="A28" s="7" t="str">
-        <x:v>FP-17</x:v>
-      </x:c>
-      <x:c r="B28" s="8" t="s">
+      <x:c r="C28" s="4"/>
+    </x:row>
+    <x:row r="29" ht="73" customHeight="1">
+      <x:c r="A29" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="35" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="C28" s="6" t="s">
+      <x:c r="C29" s="36" t="s">
         <x:v>43</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="59" customHeight="1">
-      <x:c r="A29" s="10" t="str">
-        <x:v>FP-18</x:v>
-      </x:c>
-      <x:c r="B29" s="11" t="s">
+    <x:row r="30" ht="59" customHeight="1">
+      <x:c r="A30" s="37" t="inlineStr">
+        <x:is>
+          <x:t>FP-19</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="38" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="C29" s="9" t="s">
+      <x:c r="C30" s="39" t="s">
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="59" customHeight="1">
-      <x:c r="A30" s="7" t="str">
-        <x:v>FP-19</x:v>
-      </x:c>
-      <x:c r="B30" s="8" t="s">
+    <x:row r="31" ht="59" customHeight="1">
+      <x:c r="A31" s="34" t="inlineStr">
+        <x:is>
+          <x:t>FP-20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" s="35" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="C30" s="6" t="s">
+      <x:c r="C31" s="36" t="s">
         <x:v>47</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="59" customHeight="1">
-      <x:c r="A31" s="22" t="str">
-        <x:v>FP-20</x:v>
-      </x:c>
-      <x:c r="B31" s="23" t="s">
+    <x:row r="32" ht="100.0" customHeight="1">
+      <x:c r="A32" s="40" t="inlineStr">
+        <x:is>
+          <x:t>FP-21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="41" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="C31" s="24" t="str">
-        <x:v>Pokud pro výpočet vzdálenosti chybějí potřebné údaje nebo jsou stavy tachometru rozporné, aplikace musí místo výsledku zobrazit informaci, proč výpočet nelze provést.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="59" customHeight="1">
-      <x:c r="A32" s="25" t="str">
-        <x:v>FP-21</x:v>
-      </x:c>
-      <x:c r="B32" s="26" t="s">
+      <x:c r="C32" s="42" t="inlineStr">
+        <x:is>
+          <x:t>Pokud pro výpočet vzdálenosti chybějí potřebné údaje nebo jsou stavy tachometru rozporné, aplikace musí místo výsledku zobrazit informaci, proč výpočet nelze provést. Pokud nejsou splněny podmínky výpočtu spotřeby podle FP-27, musí místo spotřeby zobrazit důvod její nedostupnosti.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="85.0" customHeight="1">
+      <x:c r="A33" s="43" t="inlineStr">
+        <x:is>
+          <x:t>FP-22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="44" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="C32" s="27" t="s">
-        <x:v>50</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="27" customHeight="1">
-      <x:c r="A33" s="20"/>
-      <x:c r="B33" s="21" t="s">
+      <x:c r="C33" s="45" t="inlineStr">
+        <x:is>
+          <x:t>Po přidání, úpravě nebo odstranění záznamů musí aplikace aktualizovat související statistiky a grafy včetně vypočtené spotřeby tak, aby odpovídaly aktuálním datům. Přepočet musí zahrnout i změnu označení tankování do plna.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="175" customHeight="1">
+      <x:c r="A34" s="40" t="inlineStr">
+        <x:is>
+          <x:t>FP-27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="41" t="inlineStr">
+        <x:is>
+          <x:t>Průměrná spotřeba vozidla</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="42" t="inlineStr">
+        <x:is>
+          <x:t>Aplikace musí pro vybrané vozidlo zobrazit průměrnou spotřebu v l/100 km za každý uzavřený úsek mezi dvěma časově po sobě následujícími tankováními označenými jako tankování do plna. U obou krajních záznamů musí být vyplněn stav tachometru a koncový stav musí být vyšší než počáteční. Do výpočtu zahrne všechna evidovaná tankování po počátečním záznamu až po koncový včetně; množství z počátečního tankování nezahrne. Mezilehlá částečná tankování nemusejí mít vyplněný tachometr. U výsledku zobrazí počáteční a koncové datum a ujetou vzdálenost. Výpočet předpokládá evidenci všech tankování v daném úseku.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="27" customHeight="1">
+      <x:c r="A35" s="20"/>
+      <x:c r="B35" s="21" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C33" s="20"/>
-    </x:row>
-    <x:row r="34" ht="59" customHeight="1">
-      <x:c r="A34" s="14" t="str">
-        <x:v>FP-22</x:v>
-      </x:c>
-      <x:c r="B34" s="15" t="s">
+      <x:c r="C35" s="20"/>
+    </x:row>
+    <x:row r="36" ht="59" customHeight="1">
+      <x:c r="A36" s="46" t="inlineStr">
+        <x:is>
+          <x:t>FP-23</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="47" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="C34" s="16" t="s">
+      <x:c r="C36" s="48" t="s">
         <x:v>53</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="59" customHeight="1">
-      <x:c r="A35" s="17" t="str">
-        <x:v>FP-23</x:v>
-      </x:c>
-      <x:c r="B35" s="18" t="s">
+    <x:row r="37" ht="59" customHeight="1">
+      <x:c r="A37" s="49" t="inlineStr">
+        <x:is>
+          <x:t>FP-24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="50" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="C35" s="19" t="s">
+      <x:c r="C37" s="51" t="s">
         <x:v>55</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="59" customHeight="1">
-      <x:c r="A36" s="14" t="str">
-        <x:v>FP-24</x:v>
-      </x:c>
-      <x:c r="B36" s="15" t="s">
+    <x:row r="38" ht="59" customHeight="1">
+      <x:c r="A38" s="46" t="inlineStr">
+        <x:is>
+          <x:t>FP-25</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="47" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="C36" s="16" t="s">
+      <x:c r="C38" s="48" t="s">
         <x:v>57</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="46" customHeight="1">
-      <x:c r="A37" s="17" t="str">
-        <x:v>FP-25</x:v>
-      </x:c>
-      <x:c r="B37" s="18" t="s">
+    <x:row r="39" ht="46" customHeight="1">
+      <x:c r="A39" s="49" t="inlineStr">
+        <x:is>
+          <x:t>FP-26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="50" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="C37" s="19" t="s">
+      <x:c r="C39" s="51" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="15" customHeight="1">
-      <x:c r="A38"/>
-      <x:c r="B38"/>
-      <x:c r="C38"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="1"/>
-      <x:c r="B39" s="1"/>
-      <x:c r="C39" s="1"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="1"/>
-      <x:c r="B40" s="1"/>
-      <x:c r="C40" s="1"/>
+    <x:row r="40" ht="15" customHeight="1">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="1"/>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="1"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="1"/>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="1"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>